<commit_message>
refactor: Alterei a página de armas para exibi-las com seus valores por tier
</commit_message>
<xml_diff>
--- a/app/data/weapons.xlsx
+++ b/app/data/weapons.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RPG\Archivum\Streamlit\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966D94B9-5D55-411F-8E70-AE51D324713F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B13804-C3A6-488D-9CF1-74D616CBC24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="265">
   <si>
     <t>weapon_id</t>
   </si>
@@ -408,9 +408,6 @@
     <t>LANÇA</t>
   </si>
   <si>
-    <t>Acrescentando-seuma ponta metálica à lança de mão sem ponta, chegamos a esta.É uma ponta simples, não muito firme, que pode facilmete ser encontrada nas civilizações que atingiram a Idade do Bronze.</t>
-  </si>
-  <si>
     <t>Pike</t>
   </si>
   <si>
@@ -771,9 +768,6 @@
     <t>weapon_tr</t>
   </si>
   <si>
-    <t>weapon_munition_price</t>
-  </si>
-  <si>
     <t>Trata-se, apenas e tão somente de um gancho.  É uma arma curta e pouco versátil, mas pode machucar muito um inimigo com um golpe no abdômem.</t>
   </si>
   <si>
@@ -823,6 +817,21 @@
   </si>
   <si>
     <t>São as tão temidas "estrelinhas dos ninjas". Trata-se de pequenos mísseis metálicos com quatro a oito pontas utilizadas como arma à distância. Não costumam matar, salvo golpes em locais precisos ou quando impregnadas em veneno.</t>
+  </si>
+  <si>
+    <t>Contusão, Perfuração</t>
+  </si>
+  <si>
+    <t>Katana</t>
+  </si>
+  <si>
+    <t>A katana é a espada dos samurais. Ela era confeccionada exclusivamente para uso do dono. Suas medidas eram projetadas para o corpo do samurai. Isto fazia dela uma arma única. Era construída com aço da mais alta qualidade existente e forjada centenas de vezes de modo a garantir altíssima resitência. Sua utilização envolve diversos procedimentos e rituais. O simples toque em uma lâmina significa a morte para quem o fez. Pode ser empunhada com uma ou duas mãos.</t>
+  </si>
+  <si>
+    <t>Acrescentando-se uma ponta metálica à lança de mão sem ponta, chegamos a esta. É uma ponta simples, não muito firme, que pode facilmete ser encontrada nas civilizações que atingiram a Idade do Bronze.</t>
+  </si>
+  <si>
+    <t>weapon_ammo_price</t>
   </si>
 </sst>
 </file>
@@ -1198,7 +1207,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z1001"/>
+  <dimension ref="A1:Z1002"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.42578125" style="8" customWidth="1"/>
@@ -1303,7 +1312,7 @@
         <v>16</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
@@ -1322,7 +1331,7 @@
     </row>
     <row r="3" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="str">
-        <f t="shared" ref="A3:A73" si="0">LEFT(A2, 6) &amp; TEXT(VALUE(RIGHT(A2, 2)) + 1, "00")</f>
+        <f t="shared" ref="A3:A74" si="0">LEFT(A2, 6) &amp; TEXT(VALUE(RIGHT(A2, 2)) + 1, "00")</f>
         <v>melee-01</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1356,7 +1365,7 @@
         <v>16</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -1391,7 +1400,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="1">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G4" s="1">
         <v>3</v>
@@ -1406,7 +1415,7 @@
         <v>6</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>20</v>
+        <v>260</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>21</v>
@@ -3069,7 +3078,7 @@
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
     </row>
-    <row r="36" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:26" ht="120" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-34</v>
@@ -3078,34 +3087,34 @@
         <v>64</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>103</v>
+        <v>261</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>97</v>
       </c>
       <c r="E36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36" s="1">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H36" s="1">
-        <v>150</v>
+        <v>1000</v>
       </c>
       <c r="I36" s="1">
         <v>1.1000000000000001</v>
       </c>
       <c r="J36" s="22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K36" s="1" t="s">
         <v>16</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>104</v>
+        <v>262</v>
       </c>
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
@@ -3122,43 +3131,43 @@
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
     </row>
-    <row r="37" spans="1:26" ht="60" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>105</v>
+        <v>64</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="E37" s="1">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="F37" s="1">
-        <v>-1</v>
-      </c>
-      <c r="G37" s="2">
-        <v>0.25</v>
+        <v>1</v>
+      </c>
+      <c r="G37" s="1">
+        <v>3</v>
       </c>
       <c r="H37" s="1">
-        <v>10</v>
-      </c>
-      <c r="I37" s="3">
-        <v>0.35</v>
+        <v>150</v>
+      </c>
+      <c r="I37" s="1">
+        <v>1.1000000000000001</v>
       </c>
       <c r="J37" s="22">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K37" s="1" t="s">
         <v>16</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
@@ -3175,7 +3184,7 @@
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
     </row>
-    <row r="38" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:26" ht="60" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-36</v>
@@ -3184,22 +3193,22 @@
         <v>105</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>107</v>
       </c>
       <c r="E38" s="1">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="F38" s="1">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="G38" s="2">
         <v>0.25</v>
       </c>
       <c r="H38" s="1">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I38" s="3">
         <v>0.35</v>
@@ -3211,7 +3220,7 @@
         <v>16</v>
       </c>
       <c r="L38" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
@@ -3228,7 +3237,7 @@
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
     </row>
-    <row r="39" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-37</v>
@@ -3237,25 +3246,25 @@
         <v>105</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D39" s="1" t="s">
         <v>107</v>
       </c>
       <c r="E39" s="1">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G39" s="2">
-        <v>0.15</v>
+        <v>0.25</v>
       </c>
       <c r="H39" s="1">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="I39" s="3">
-        <v>0.25</v>
+        <v>0.35</v>
       </c>
       <c r="J39" s="22">
         <v>6</v>
@@ -3264,7 +3273,7 @@
         <v>16</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
@@ -3281,7 +3290,7 @@
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
     </row>
-    <row r="40" spans="1:26" ht="60" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-38</v>
@@ -3290,7 +3299,7 @@
         <v>105</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D40" s="1" t="s">
         <v>107</v>
@@ -3299,16 +3308,16 @@
         <v>-1</v>
       </c>
       <c r="F40" s="1">
-        <v>1</v>
-      </c>
-      <c r="G40" s="1">
+        <v>3</v>
+      </c>
+      <c r="G40" s="2">
         <v>0.15</v>
       </c>
       <c r="H40" s="1">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="I40" s="3">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="J40" s="22">
         <v>6</v>
@@ -3317,7 +3326,7 @@
         <v>16</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
@@ -3334,7 +3343,7 @@
       <c r="Y40" s="1"/>
       <c r="Z40" s="1"/>
     </row>
-    <row r="41" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:26" ht="60" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-39</v>
@@ -3343,25 +3352,25 @@
         <v>105</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>107</v>
       </c>
       <c r="E41" s="1">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="F41" s="1">
         <v>1</v>
       </c>
       <c r="G41" s="1">
-        <v>1.4</v>
+        <v>0.15</v>
       </c>
       <c r="H41" s="1">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I41" s="3">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="J41" s="22">
         <v>6</v>
@@ -3370,7 +3379,7 @@
         <v>16</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
@@ -3396,7 +3405,7 @@
         <v>105</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>107</v>
@@ -3405,25 +3414,25 @@
         <v>2</v>
       </c>
       <c r="F42" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G42" s="1">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
       <c r="H42" s="1">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="I42" s="3">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="J42" s="22">
         <v>6</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
@@ -3449,7 +3458,7 @@
         <v>105</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>107</v>
@@ -3458,25 +3467,25 @@
         <v>2</v>
       </c>
       <c r="F43" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G43" s="1">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="H43" s="1">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="I43" s="3">
-        <v>0.28000000000000003</v>
+        <v>0.45</v>
       </c>
       <c r="J43" s="22">
         <v>6</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M43" s="1"/>
       <c r="N43" s="1"/>
@@ -3493,43 +3502,43 @@
       <c r="Y43" s="1"/>
       <c r="Z43" s="1"/>
     </row>
-    <row r="44" spans="1:26" ht="60" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-42</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>121</v>
+        <v>105</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="E44" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F44" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G44" s="1">
-        <v>2</v>
+        <v>0.35</v>
       </c>
       <c r="H44" s="1">
-        <v>50</v>
-      </c>
-      <c r="I44" s="1">
-        <v>1.5</v>
+        <v>200</v>
+      </c>
+      <c r="I44" s="3">
+        <v>0.28000000000000003</v>
       </c>
       <c r="J44" s="22">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
@@ -3546,7 +3555,7 @@
       <c r="Y44" s="1"/>
       <c r="Z44" s="1"/>
     </row>
-    <row r="45" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:26" ht="60" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-43</v>
@@ -3555,7 +3564,7 @@
         <v>121</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>123</v>
@@ -3564,25 +3573,25 @@
         <v>0</v>
       </c>
       <c r="F45" s="1">
+        <v>1</v>
+      </c>
+      <c r="G45" s="1">
         <v>2</v>
       </c>
-      <c r="G45" s="1">
-        <v>2.5</v>
-      </c>
       <c r="H45" s="1">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="I45" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J45" s="22">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K45" s="1" t="s">
         <v>47</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>126</v>
+        <v>263</v>
       </c>
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
@@ -3599,7 +3608,7 @@
       <c r="Y45" s="1"/>
       <c r="Z45" s="1"/>
     </row>
-    <row r="46" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-44</v>
@@ -3608,7 +3617,7 @@
         <v>121</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>123</v>
@@ -3623,10 +3632,10 @@
         <v>2.5</v>
       </c>
       <c r="H46" s="1">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="I46" s="1">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="J46" s="22">
         <v>9</v>
@@ -3635,7 +3644,7 @@
         <v>47</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
@@ -3661,7 +3670,7 @@
         <v>121</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>123</v>
@@ -3670,25 +3679,25 @@
         <v>0</v>
       </c>
       <c r="F47" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G47" s="1">
         <v>2.5</v>
       </c>
       <c r="H47" s="1">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="I47" s="1">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="J47" s="22">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K47" s="1" t="s">
         <v>47</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="M47" s="1"/>
       <c r="N47" s="1"/>
@@ -3714,7 +3723,7 @@
         <v>121</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D48" s="1" t="s">
         <v>123</v>
@@ -3726,22 +3735,22 @@
         <v>1</v>
       </c>
       <c r="G48" s="1">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="H48" s="1">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="I48" s="1">
         <v>1.5</v>
       </c>
       <c r="J48" s="22">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K48" s="1" t="s">
         <v>47</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
@@ -3767,7 +3776,7 @@
         <v>121</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>123</v>
@@ -3776,13 +3785,13 @@
         <v>0</v>
       </c>
       <c r="F49" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49" s="1">
         <v>2</v>
       </c>
       <c r="H49" s="1">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="I49" s="1">
         <v>1.5</v>
@@ -3794,7 +3803,7 @@
         <v>47</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
@@ -3811,7 +3820,7 @@
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
     </row>
-    <row r="50" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-48</v>
@@ -3820,7 +3829,7 @@
         <v>121</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>123</v>
@@ -3829,25 +3838,25 @@
         <v>0</v>
       </c>
       <c r="F50" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G50" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H50" s="1">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="I50" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J50" s="22">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K50" s="1" t="s">
         <v>47</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
@@ -3864,7 +3873,7 @@
       <c r="Y50" s="1"/>
       <c r="Z50" s="1"/>
     </row>
-    <row r="51" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-49</v>
@@ -3873,7 +3882,7 @@
         <v>121</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D51" s="1" t="s">
         <v>123</v>
@@ -3882,25 +3891,25 @@
         <v>0</v>
       </c>
       <c r="F51" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G51" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H51" s="1">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="I51" s="1">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="J51" s="22">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="K51" s="1" t="s">
         <v>47</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
@@ -3917,7 +3926,7 @@
       <c r="Y51" s="1"/>
       <c r="Z51" s="1"/>
     </row>
-    <row r="52" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-50</v>
@@ -3926,7 +3935,7 @@
         <v>121</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D52" s="1" t="s">
         <v>123</v>
@@ -3935,25 +3944,25 @@
         <v>0</v>
       </c>
       <c r="F52" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G52" s="1">
-        <v>7.5</v>
+        <v>4</v>
       </c>
       <c r="H52" s="1">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="I52" s="1">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="J52" s="22">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K52" s="1" t="s">
         <v>47</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
@@ -3970,43 +3979,43 @@
       <c r="Y52" s="1"/>
       <c r="Z52" s="1"/>
     </row>
-    <row r="53" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-51</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>141</v>
+        <v>121</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="E53" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F53" s="1">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G53" s="1">
-        <v>3</v>
+        <v>7.5</v>
       </c>
       <c r="H53" s="1">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="I53" s="1">
-        <v>0.6</v>
+        <v>4</v>
       </c>
       <c r="J53" s="22">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
@@ -4023,31 +4032,31 @@
       <c r="Y53" s="1"/>
       <c r="Z53" s="1"/>
     </row>
-    <row r="54" spans="1:26" ht="84" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-52</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C54" s="1" t="s">
-        <v>145</v>
-      </c>
       <c r="D54" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E54" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F54" s="1">
         <v>0</v>
       </c>
       <c r="G54" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H54" s="1">
-        <v>230</v>
+        <v>80</v>
       </c>
       <c r="I54" s="1">
         <v>0.6</v>
@@ -4059,7 +4068,7 @@
         <v>32</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="M54" s="1"/>
       <c r="N54" s="1"/>
@@ -4076,22 +4085,22 @@
       <c r="Y54" s="1"/>
       <c r="Z54" s="1"/>
     </row>
-    <row r="55" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:26" ht="84" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-53</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E55" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F55" s="1">
         <v>0</v>
@@ -4100,19 +4109,19 @@
         <v>4</v>
       </c>
       <c r="H55" s="1">
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="I55" s="1">
         <v>0.6</v>
       </c>
       <c r="J55" s="22">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K55" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="M55" s="1"/>
       <c r="N55" s="1"/>
@@ -4129,43 +4138,43 @@
       <c r="Y55" s="1"/>
       <c r="Z55" s="1"/>
     </row>
-    <row r="56" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-54</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E56" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F56" s="1">
         <v>0</v>
       </c>
       <c r="G56" s="1">
-        <v>1.2</v>
+        <v>4</v>
       </c>
       <c r="H56" s="1">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="I56" s="1">
-        <v>0.45</v>
+        <v>0.6</v>
       </c>
       <c r="J56" s="22">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K56" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="M56" s="1"/>
       <c r="N56" s="1"/>
@@ -4188,37 +4197,37 @@
         <v>melee-55</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E57" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F57" s="1">
         <v>0</v>
       </c>
       <c r="G57" s="1">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="H57" s="1">
-        <v>200</v>
+        <v>70</v>
       </c>
       <c r="I57" s="1">
-        <v>0.55000000000000004</v>
+        <v>0.45</v>
       </c>
       <c r="J57" s="22">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K57" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="M57" s="1"/>
       <c r="N57" s="1"/>
@@ -4235,19 +4244,19 @@
       <c r="Y57" s="1"/>
       <c r="Z57" s="1"/>
     </row>
-    <row r="58" spans="1:26" ht="60" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-56</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>154</v>
+        <v>150</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>142</v>
       </c>
       <c r="E58" s="1">
         <v>2</v>
@@ -4256,22 +4265,22 @@
         <v>0</v>
       </c>
       <c r="G58" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H58" s="1">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="I58" s="1">
-        <v>1</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="J58" s="22">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="K58" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="M58" s="1"/>
       <c r="N58" s="1"/>
@@ -4288,22 +4297,22 @@
       <c r="Y58" s="1"/>
       <c r="Z58" s="1"/>
     </row>
-    <row r="59" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:26" ht="60" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-57</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E59" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59" s="1">
         <v>0</v>
@@ -4312,19 +4321,19 @@
         <v>5</v>
       </c>
       <c r="H59" s="1">
-        <v>320</v>
+        <v>60</v>
       </c>
       <c r="I59" s="1">
-        <v>1.3</v>
+        <v>1</v>
       </c>
       <c r="J59" s="22">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K59" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="M59" s="1"/>
       <c r="N59" s="1"/>
@@ -4347,22 +4356,22 @@
         <v>melee-58</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E60" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F60" s="1">
         <v>0</v>
       </c>
       <c r="G60" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H60" s="1">
         <v>320</v>
@@ -4371,13 +4380,13 @@
         <v>1.3</v>
       </c>
       <c r="J60" s="22">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K60" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="M60" s="1"/>
       <c r="N60" s="1"/>
@@ -4400,37 +4409,37 @@
         <v>melee-59</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>160</v>
+        <v>140</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>143</v>
+        <v>157</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>153</v>
       </c>
       <c r="E61" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F61" s="1">
         <v>0</v>
       </c>
       <c r="G61" s="1">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="H61" s="1">
-        <v>25</v>
+        <v>320</v>
       </c>
       <c r="I61" s="1">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="J61" s="22">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="L61" s="1" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="M61" s="1"/>
       <c r="N61" s="1"/>
@@ -4447,22 +4456,22 @@
       <c r="Y61" s="1"/>
       <c r="Z61" s="1"/>
     </row>
-    <row r="62" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-60</v>
       </c>
       <c r="B62" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="C62" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="D62" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E62" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" s="1">
         <v>0</v>
@@ -4471,10 +4480,10 @@
         <v>1.5</v>
       </c>
       <c r="H62" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I62" s="1">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="J62" s="22">
         <v>7</v>
@@ -4483,7 +4492,7 @@
         <v>20</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="M62" s="1"/>
       <c r="N62" s="1"/>
@@ -4506,37 +4515,37 @@
         <v>melee-61</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E63" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" s="1">
         <v>0</v>
       </c>
       <c r="G63" s="1">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="H63" s="1">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="I63" s="1">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="J63" s="22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K63" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="M63" s="1"/>
       <c r="N63" s="1"/>
@@ -4553,43 +4562,43 @@
       <c r="Y63" s="1"/>
       <c r="Z63" s="1"/>
     </row>
-    <row r="64" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-62</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E64" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F64" s="1">
         <v>0</v>
       </c>
       <c r="G64" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H64" s="1">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="I64" s="1">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="J64" s="22">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K64" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L64" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="M64" s="1"/>
       <c r="N64" s="1"/>
@@ -4612,37 +4621,37 @@
         <v>melee-63</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E65" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F65" s="1">
         <v>0</v>
       </c>
       <c r="G65" s="1">
+        <v>5</v>
+      </c>
+      <c r="H65" s="1">
+        <v>100</v>
+      </c>
+      <c r="I65" s="1">
         <v>1</v>
       </c>
-      <c r="H65" s="1">
-        <v>20</v>
-      </c>
-      <c r="I65" s="1">
-        <v>0.5</v>
-      </c>
       <c r="J65" s="22">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="K65" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L65" s="1" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="M65" s="1"/>
       <c r="N65" s="1"/>
@@ -4659,43 +4668,43 @@
       <c r="Y65" s="1"/>
       <c r="Z65" s="1"/>
     </row>
-    <row r="66" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-64</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>173</v>
+        <v>142</v>
       </c>
       <c r="E66" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F66" s="1">
         <v>0</v>
       </c>
       <c r="G66" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H66" s="1">
-        <v>100</v>
-      </c>
-      <c r="I66" s="10">
+        <v>20</v>
+      </c>
+      <c r="I66" s="1">
         <v>0.5</v>
       </c>
       <c r="J66" s="22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K66" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="M66" s="1"/>
       <c r="N66" s="1"/>
@@ -4718,37 +4727,37 @@
         <v>melee-65</v>
       </c>
       <c r="B67" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C67" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="C67" s="1" t="s">
-        <v>175</v>
-      </c>
       <c r="D67" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E67" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F67" s="1">
         <v>0</v>
       </c>
       <c r="G67" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H67" s="1">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="I67" s="10">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="J67" s="22">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="K67" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="M67" s="1"/>
       <c r="N67" s="1"/>
@@ -4771,16 +4780,16 @@
         <v>melee-66</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E68" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F68" s="1">
         <v>0</v>
@@ -4789,19 +4798,19 @@
         <v>5</v>
       </c>
       <c r="H68" s="1">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="I68" s="10">
         <v>1</v>
       </c>
       <c r="J68" s="22">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K68" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="M68" s="1"/>
       <c r="N68" s="1"/>
@@ -4824,37 +4833,37 @@
         <v>melee-67</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E69" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F69" s="1">
         <v>0</v>
       </c>
       <c r="G69" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H69" s="1">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I69" s="10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J69" s="22">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K69" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L69" s="1" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="M69" s="1"/>
       <c r="N69" s="1"/>
@@ -4877,37 +4886,37 @@
         <v>melee-68</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>143</v>
+        <v>172</v>
       </c>
       <c r="E70" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F70" s="1">
         <v>0</v>
       </c>
       <c r="G70" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H70" s="1">
-        <v>25</v>
-      </c>
-      <c r="I70" s="1">
-        <v>0.8</v>
+        <v>200</v>
+      </c>
+      <c r="I70" s="10">
+        <v>2</v>
       </c>
       <c r="J70" s="22">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K70" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L70" s="1" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="M70" s="1"/>
       <c r="N70" s="1"/>
@@ -4924,43 +4933,43 @@
       <c r="Y70" s="1"/>
       <c r="Z70" s="1"/>
     </row>
-    <row r="71" spans="1:26" ht="48" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:26" ht="36" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-69</v>
       </c>
       <c r="B71" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="C71" s="1" t="s">
-        <v>184</v>
-      </c>
       <c r="D71" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E71" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F71" s="1">
         <v>0</v>
       </c>
       <c r="G71" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H71" s="1">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="I71" s="1">
         <v>0.8</v>
       </c>
       <c r="J71" s="22">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K71" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="M71" s="1"/>
       <c r="N71" s="1"/>
@@ -4977,43 +4986,43 @@
       <c r="Y71" s="1"/>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" spans="1:26" ht="60" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:26" ht="48" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-70</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>125</v>
+        <v>183</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="E72" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F72" s="1">
         <v>0</v>
       </c>
       <c r="G72" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H72" s="1">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="I72" s="1">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="J72" s="22">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K72" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L72" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="M72" s="1"/>
       <c r="N72" s="1"/>
@@ -5030,43 +5039,43 @@
       <c r="Y72" s="1"/>
       <c r="Z72" s="1"/>
     </row>
-    <row r="73" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:26" ht="60" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="str">
         <f t="shared" si="0"/>
         <v>melee-71</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>187</v>
+        <v>124</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E73" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F73" s="1">
         <v>0</v>
       </c>
       <c r="G73" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H73" s="1">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="I73" s="1">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J73" s="22">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K73" s="1" t="s">
         <v>20</v>
       </c>
       <c r="L73" s="1" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="M73" s="1"/>
       <c r="N73" s="1"/>
@@ -5083,19 +5092,44 @@
       <c r="Y73" s="1"/>
       <c r="Z73" s="1"/>
     </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A74" s="1"/>
-      <c r="B74" s="1"/>
-      <c r="C74" s="1"/>
-      <c r="D74" s="1"/>
-      <c r="E74" s="1"/>
-      <c r="F74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="1"/>
-      <c r="I74" s="1"/>
-      <c r="J74" s="22"/>
-      <c r="K74" s="1"/>
-      <c r="L74" s="1"/>
+    <row r="74" spans="1:26" ht="36" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>melee-72</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E74" s="1">
+        <v>5</v>
+      </c>
+      <c r="F74" s="1">
+        <v>0</v>
+      </c>
+      <c r="G74" s="1">
+        <v>8</v>
+      </c>
+      <c r="H74" s="1">
+        <v>100</v>
+      </c>
+      <c r="I74" s="1">
+        <v>2</v>
+      </c>
+      <c r="J74" s="22">
+        <v>14</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="L74" s="1" t="s">
+        <v>187</v>
+      </c>
       <c r="M74" s="1"/>
       <c r="N74" s="1"/>
       <c r="O74" s="1"/>
@@ -31066,6 +31100,34 @@
       <c r="X1001" s="1"/>
       <c r="Y1001" s="1"/>
       <c r="Z1001" s="1"/>
+    </row>
+    <row r="1002" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A1002" s="1"/>
+      <c r="B1002" s="1"/>
+      <c r="C1002" s="1"/>
+      <c r="D1002" s="1"/>
+      <c r="E1002" s="1"/>
+      <c r="F1002" s="1"/>
+      <c r="G1002" s="1"/>
+      <c r="H1002" s="1"/>
+      <c r="I1002" s="1"/>
+      <c r="J1002" s="22"/>
+      <c r="K1002" s="1"/>
+      <c r="L1002" s="1"/>
+      <c r="M1002" s="1"/>
+      <c r="N1002" s="1"/>
+      <c r="O1002" s="1"/>
+      <c r="P1002" s="1"/>
+      <c r="Q1002" s="1"/>
+      <c r="R1002" s="1"/>
+      <c r="S1002" s="1"/>
+      <c r="T1002" s="1"/>
+      <c r="U1002" s="1"/>
+      <c r="V1002" s="1"/>
+      <c r="W1002" s="1"/>
+      <c r="X1002" s="1"/>
+      <c r="Y1002" s="1"/>
+      <c r="Z1002" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -31123,7 +31185,7 @@
         <v>7</v>
       </c>
       <c r="H1" s="15" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="I1" s="11" t="s">
         <v>8</v>
@@ -31135,19 +31197,19 @@
         <v>10</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="N1" s="11" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O1" s="11" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="P1" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="Q1" s="11" t="s">
         <v>11</v>
@@ -31169,16 +31231,16 @@
     </row>
     <row r="2" spans="1:31" ht="24" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>106</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E2" s="6">
         <v>1</v>
@@ -31189,9 +31251,7 @@
       <c r="G2" s="6">
         <v>10</v>
       </c>
-      <c r="H2" s="14">
-        <v>10</v>
-      </c>
+      <c r="H2" s="14"/>
       <c r="I2" s="6">
         <v>0.3</v>
       </c>
@@ -31208,16 +31268,16 @@
         <v>1</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="R2" s="5"/>
       <c r="S2" s="5"/>
@@ -31240,13 +31300,13 @@
         <v>ranged-01</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E3" s="6">
         <v>1</v>
@@ -31257,17 +31317,15 @@
       <c r="G3" s="12">
         <v>70</v>
       </c>
-      <c r="H3" s="14">
-        <v>70</v>
-      </c>
+      <c r="H3" s="14"/>
       <c r="I3" s="12">
         <v>0.45</v>
       </c>
       <c r="J3" s="18">
         <v>7</v>
       </c>
-      <c r="K3" s="13" t="s">
-        <v>32</v>
+      <c r="K3" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="L3" s="6">
         <v>11</v>
@@ -31276,16 +31334,16 @@
         <v>1</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q3" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="R3" s="5"/>
       <c r="S3" s="5"/>
@@ -31308,13 +31366,13 @@
         <v>ranged-02</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E4" s="6">
         <v>1</v>
@@ -31325,17 +31383,15 @@
       <c r="G4" s="12">
         <v>200</v>
       </c>
-      <c r="H4" s="14">
-        <v>200</v>
-      </c>
+      <c r="H4" s="14"/>
       <c r="I4" s="12">
         <v>0.55000000000000004</v>
       </c>
       <c r="J4" s="18">
         <v>10</v>
       </c>
-      <c r="K4" s="13" t="s">
-        <v>32</v>
+      <c r="K4" s="6" t="s">
+        <v>47</v>
       </c>
       <c r="L4" s="6">
         <v>10</v>
@@ -31344,16 +31400,16 @@
         <v>2</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O4" s="6" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q4" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="R4" s="5"/>
       <c r="S4" s="5"/>
@@ -31376,13 +31432,13 @@
         <v>ranged-03</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E5" s="6">
         <v>0</v>
@@ -31412,16 +31468,16 @@
         <v>1</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="R5" s="5"/>
       <c r="S5" s="5"/>
@@ -31444,13 +31500,13 @@
         <v>ranged-04</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E6" s="6">
         <v>2</v>
@@ -31480,16 +31536,16 @@
         <v>3</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="R6" s="5"/>
       <c r="S6" s="5"/>
@@ -31512,13 +31568,13 @@
         <v>ranged-05</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>228</v>
-      </c>
       <c r="D7" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E7" s="6">
         <v>3</v>
@@ -31548,16 +31604,16 @@
         <v>3</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="R7" s="5"/>
       <c r="S7" s="5"/>
@@ -31580,13 +31636,13 @@
         <v>ranged-06</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E8" s="6">
         <v>4</v>
@@ -31616,16 +31672,16 @@
         <v>4</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="R8" s="5"/>
       <c r="S8" s="5"/>
@@ -31648,13 +31704,13 @@
         <v>ranged-07</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E9" s="6">
         <v>2</v>
@@ -31684,16 +31740,16 @@
         <v>4</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="R9" s="5"/>
       <c r="S9" s="5"/>
@@ -31716,13 +31772,13 @@
         <v>ranged-08</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E10" s="6">
         <v>3</v>
@@ -31752,16 +31808,16 @@
         <v>4</v>
       </c>
       <c r="N10" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
@@ -31784,13 +31840,13 @@
         <v>ranged-09</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E11" s="6">
         <v>1</v>
@@ -31820,16 +31876,16 @@
         <v>2</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="R11" s="5"/>
       <c r="S11" s="5"/>
@@ -31852,13 +31908,13 @@
         <v>ranged-10</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E12" s="6">
         <v>4</v>
@@ -31888,16 +31944,16 @@
         <v>2</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="R12" s="5"/>
       <c r="S12" s="5"/>
@@ -31920,13 +31976,13 @@
         <v>ranged-11</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>122</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E13" s="6">
         <v>1</v>
@@ -31956,16 +32012,16 @@
         <v>1</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>124</v>
+        <v>263</v>
       </c>
       <c r="R13" s="5"/>
       <c r="S13" s="5"/>
@@ -31988,13 +32044,13 @@
         <v>ranged-12</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E14" s="6">
         <v>2</v>
@@ -32015,7 +32071,7 @@
         <v>7</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L14" s="6">
         <v>12</v>
@@ -32024,16 +32080,16 @@
         <v>2</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="Q14" s="6" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="R14" s="5"/>
       <c r="S14" s="5"/>
@@ -32059,10 +32115,10 @@
         <v>13</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E15" s="6">
         <v>1</v>
@@ -32092,16 +32148,16 @@
         <v>1</v>
       </c>
       <c r="N15" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="R15" s="5"/>
       <c r="S15" s="5"/>
@@ -32127,10 +32183,10 @@
         <v>13</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E16" s="6">
         <v>1</v>
@@ -32160,16 +32216,16 @@
         <v>1</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="R16" s="5"/>
       <c r="S16" s="5"/>
@@ -32195,10 +32251,10 @@
         <v>13</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E17" s="6">
         <v>0</v>
@@ -32228,16 +32284,16 @@
         <v>1</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="P17" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="R17" s="5"/>
       <c r="S17" s="5"/>
@@ -32263,10 +32319,10 @@
         <v>13</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E18" s="6">
         <v>1</v>
@@ -32277,9 +32333,7 @@
       <c r="G18" s="6">
         <v>80</v>
       </c>
-      <c r="H18" s="14">
-        <v>80</v>
-      </c>
+      <c r="H18" s="14"/>
       <c r="I18" s="6">
         <v>0.45</v>
       </c>
@@ -32296,16 +32350,16 @@
         <v>1</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="R18" s="5"/>
       <c r="S18" s="5"/>
@@ -32331,10 +32385,10 @@
         <v>13</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E19" s="6">
         <v>0</v>
@@ -32345,9 +32399,7 @@
       <c r="G19" s="6">
         <v>100</v>
       </c>
-      <c r="H19" s="6">
-        <v>100</v>
-      </c>
+      <c r="H19" s="6"/>
       <c r="I19" s="6">
         <v>2</v>
       </c>
@@ -32364,16 +32416,16 @@
         <v>1</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="R19" s="5"/>
       <c r="S19" s="5"/>
@@ -32399,10 +32451,10 @@
         <v>13</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E20" s="6">
         <v>1</v>
@@ -32413,9 +32465,7 @@
       <c r="G20" s="6">
         <v>10</v>
       </c>
-      <c r="H20" s="14">
-        <v>10</v>
-      </c>
+      <c r="H20" s="14"/>
       <c r="I20" s="6">
         <v>0.1</v>
       </c>
@@ -32432,16 +32482,16 @@
         <v>0</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="R20" s="5"/>
       <c r="S20" s="5"/>

</xml_diff>

<commit_message>
add: Adicionei novas entradas nas bases de armas
</commit_message>
<xml_diff>
--- a/app/data/weapons.xlsx
+++ b/app/data/weapons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RPG\Archivum\Streamlit\app\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B13804-C3A6-488D-9CF1-74D616CBC24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A081F0A-96DF-4B40-B305-8A02B9928CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="melee" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="272">
   <si>
     <t>weapon_id</t>
   </si>
@@ -833,6 +833,27 @@
   <si>
     <t>weapon_ammo_price</t>
   </si>
+  <si>
+    <t>ranged-19</t>
+  </si>
+  <si>
+    <t>Mágica</t>
+  </si>
+  <si>
+    <t>Arremessar Feitiço</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>IQ x 10</t>
+  </si>
+  <si>
+    <t>IQ x 15</t>
+  </si>
+  <si>
+    <t>Magia base para feitiços do tipo Projétil.</t>
+  </si>
 </sst>
 </file>
 
@@ -31251,7 +31272,9 @@
       <c r="G2" s="6">
         <v>10</v>
       </c>
-      <c r="H2" s="14"/>
+      <c r="H2" s="14">
+        <v>0</v>
+      </c>
       <c r="I2" s="6">
         <v>0.3</v>
       </c>
@@ -31317,7 +31340,9 @@
       <c r="G3" s="12">
         <v>70</v>
       </c>
-      <c r="H3" s="14"/>
+      <c r="H3" s="14">
+        <v>0</v>
+      </c>
       <c r="I3" s="12">
         <v>0.45</v>
       </c>
@@ -31383,7 +31408,9 @@
       <c r="G4" s="12">
         <v>200</v>
       </c>
-      <c r="H4" s="14"/>
+      <c r="H4" s="14">
+        <v>0</v>
+      </c>
       <c r="I4" s="12">
         <v>0.55000000000000004</v>
       </c>
@@ -32333,7 +32360,9 @@
       <c r="G18" s="6">
         <v>80</v>
       </c>
-      <c r="H18" s="14"/>
+      <c r="H18" s="14">
+        <v>0</v>
+      </c>
       <c r="I18" s="6">
         <v>0.45</v>
       </c>
@@ -32399,7 +32428,9 @@
       <c r="G19" s="6">
         <v>100</v>
       </c>
-      <c r="H19" s="6"/>
+      <c r="H19" s="6">
+        <v>0</v>
+      </c>
       <c r="I19" s="6">
         <v>2</v>
       </c>
@@ -32465,7 +32496,9 @@
       <c r="G20" s="6">
         <v>10</v>
       </c>
-      <c r="H20" s="14"/>
+      <c r="H20" s="14">
+        <v>0</v>
+      </c>
       <c r="I20" s="6">
         <v>0.1</v>
       </c>
@@ -32508,23 +32541,58 @@
       <c r="AD20" s="5"/>
       <c r="AE20" s="5"/>
     </row>
-    <row r="21" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
+    <row r="21" spans="1:31" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5">
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21" s="5">
+        <v>0</v>
+      </c>
+      <c r="J21" s="19">
+        <v>0</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="L21" s="5">
+        <v>12</v>
+      </c>
+      <c r="M21" s="5">
+        <v>2</v>
+      </c>
+      <c r="N21" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="O21" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="P21" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="Q21" s="5" t="s">
+        <v>271</v>
+      </c>
       <c r="R21" s="5"/>
       <c r="S21" s="5"/>
       <c r="T21" s="5"/>

</xml_diff>